<commit_message>
feat(cli): command line executable
</commit_message>
<xml_diff>
--- a/TempRegPy.xlsx
+++ b/TempRegPy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\GitHub\TempRegPy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6FB517C-80A9-4293-8E2C-DB2F24E5D815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180EFB08-0071-41B5-9496-5CE25F5602B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14205" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{EDE72A4E-5E83-4998-A3FD-57974B6FA13E}"/>
   </bookViews>
@@ -405,9 +405,6 @@
     <t>Simulation Folder Name</t>
   </si>
   <si>
-    <t>Test1</t>
-  </si>
-  <si>
     <t>Info</t>
   </si>
   <si>
@@ -424,6 +421,9 @@
   </si>
   <si>
     <t>Helpers</t>
+  </si>
+  <si>
+    <t>Test2</t>
   </si>
 </sst>
 </file>
@@ -1200,7 +1200,7 @@
     </row>
     <row r="2" spans="4:30" s="15" customFormat="1" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
       <c r="D2" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -1231,19 +1231,19 @@
     </row>
     <row r="3" spans="4:30" ht="15.75" customHeight="1" thickTop="1">
       <c r="D3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F3" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="G3" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="H3" s="19" t="s">
         <v>127</v>
       </c>
-      <c r="H3" s="19" t="s">
-        <v>128</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="AD3" s="19" t="b">
         <v>1</v>
@@ -1309,7 +1309,7 @@
         <v>120</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="4:30" ht="15.75" customHeight="1">
@@ -1579,7 +1579,7 @@
         <v>15000</v>
       </c>
       <c r="N18" s="8">
-        <v>15000</v>
+        <v>10000</v>
       </c>
       <c r="O18" s="8">
         <v>15000</v>

</xml_diff>